<commit_message>
Update program definition to be dynamic, rename to Status Quo, fix indentation
</commit_message>
<xml_diff>
--- a/data/model_parameters.xlsx
+++ b/data/model_parameters.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ravik\OneDrive\Documents\My-Projects\RabiesEcon-in-Python\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52972B82-EAF7-476A-85B4-0D8342C02101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF27A94B-9917-4BC0-9819-1A2EBEF3C2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Parameter" sheetId="1" r:id="rId1"/>
     <sheet name="Suspect animal cost parameters" sheetId="2" r:id="rId2"/>
     <sheet name="PEP costs" sheetId="4" r:id="rId3"/>
     <sheet name="Vaccination Cost" sheetId="3" r:id="rId4"/>
@@ -2153,23 +2153,14 @@
     <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2179,84 +2170,6 @@
       <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="5" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="5" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="5" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2352,6 +2265,93 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="5" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2587,7 +2587,7 @@
       <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7"/>
+      <sheetData sheetId="7" refreshError="1"/>
       <sheetData sheetId="8" refreshError="1"/>
       <sheetData sheetId="9" refreshError="1"/>
       <sheetData sheetId="10">
@@ -3895,16 +3895,16 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="174" t="s">
+      <c r="H5" s="196" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="175"/>
-      <c r="J5" s="176">
+      <c r="I5" s="197"/>
+      <c r="J5" s="198">
         <v>0.1</v>
       </c>
-      <c r="K5" s="177"/>
-      <c r="L5" s="178"/>
-      <c r="M5" s="179"/>
+      <c r="K5" s="199"/>
+      <c r="L5" s="200"/>
+      <c r="M5" s="201"/>
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -3953,30 +3953,30 @@
         <v>59</v>
       </c>
       <c r="G7" s="6"/>
-      <c r="H7" s="180" t="s">
+      <c r="H7" s="202" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="181"/>
-      <c r="J7" s="182" t="s">
+      <c r="I7" s="203"/>
+      <c r="J7" s="204" t="s">
         <v>56</v>
       </c>
-      <c r="K7" s="182"/>
-      <c r="L7" s="157" t="s">
+      <c r="K7" s="204"/>
+      <c r="L7" s="205" t="s">
         <v>61</v>
       </c>
-      <c r="M7" s="157"/>
-      <c r="N7" s="157" t="s">
+      <c r="M7" s="205"/>
+      <c r="N7" s="205" t="s">
         <v>62</v>
       </c>
-      <c r="O7" s="157"/>
-      <c r="P7" s="158"/>
+      <c r="O7" s="205"/>
+      <c r="P7" s="206"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
     </row>
     <row r="8" spans="1:20" ht="15.5" thickTop="1" x14ac:dyDescent="0.75">
-      <c r="A8" s="213" t="s">
+      <c r="A8" s="189" t="s">
         <v>63</v>
       </c>
       <c r="B8" s="17" t="s">
@@ -3996,32 +3996,32 @@
         <v>46046</v>
       </c>
       <c r="G8" s="6"/>
-      <c r="H8" s="172" t="s">
+      <c r="H8" s="191" t="s">
         <v>65</v>
       </c>
-      <c r="I8" s="173"/>
-      <c r="J8" s="159">
+      <c r="I8" s="192"/>
+      <c r="J8" s="193">
         <f>B5</f>
         <v>656500</v>
       </c>
-      <c r="K8" s="160"/>
-      <c r="L8" s="161">
+      <c r="K8" s="194"/>
+      <c r="L8" s="195">
         <v>0.53</v>
       </c>
-      <c r="M8" s="161"/>
-      <c r="N8" s="162">
+      <c r="M8" s="195"/>
+      <c r="N8" s="160">
         <f>L8*J8</f>
         <v>347945</v>
       </c>
-      <c r="O8" s="162"/>
-      <c r="P8" s="163"/>
+      <c r="O8" s="160"/>
+      <c r="P8" s="161"/>
       <c r="Q8" s="6"/>
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
       <c r="T8" s="6"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.75">
-      <c r="A9" s="199"/>
+      <c r="A9" s="175"/>
       <c r="B9" s="18" t="s">
         <v>66</v>
       </c>
@@ -4039,32 +4039,32 @@
         <v>21164</v>
       </c>
       <c r="G9" s="6"/>
-      <c r="H9" s="172" t="s">
+      <c r="H9" s="191" t="s">
         <v>67</v>
       </c>
-      <c r="I9" s="173"/>
-      <c r="J9" s="159">
+      <c r="I9" s="192"/>
+      <c r="J9" s="193">
         <f>B5</f>
         <v>656500</v>
       </c>
-      <c r="K9" s="160"/>
-      <c r="L9" s="161">
+      <c r="K9" s="194"/>
+      <c r="L9" s="195">
         <v>0.1</v>
       </c>
-      <c r="M9" s="161"/>
-      <c r="N9" s="162">
+      <c r="M9" s="195"/>
+      <c r="N9" s="160">
         <f>L9*J9</f>
         <v>65650</v>
       </c>
-      <c r="O9" s="162"/>
-      <c r="P9" s="163"/>
+      <c r="O9" s="160"/>
+      <c r="P9" s="161"/>
       <c r="Q9" s="6"/>
       <c r="R9" s="6"/>
       <c r="S9" s="6"/>
       <c r="T9" s="6"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.75">
-      <c r="A10" s="199"/>
+      <c r="A10" s="175"/>
       <c r="B10" s="18" t="s">
         <v>68</v>
       </c>
@@ -4082,32 +4082,32 @@
         <v>66466.399999999994</v>
       </c>
       <c r="G10" s="6"/>
-      <c r="H10" s="170" t="s">
+      <c r="H10" s="213" t="s">
         <v>69</v>
       </c>
-      <c r="I10" s="171"/>
-      <c r="J10" s="159">
+      <c r="I10" s="214"/>
+      <c r="J10" s="193">
         <f>B5</f>
         <v>656500</v>
       </c>
-      <c r="K10" s="160"/>
-      <c r="L10" s="161">
+      <c r="K10" s="194"/>
+      <c r="L10" s="195">
         <v>0.05</v>
       </c>
-      <c r="M10" s="161"/>
-      <c r="N10" s="162">
+      <c r="M10" s="195"/>
+      <c r="N10" s="160">
         <f>L10*J10</f>
         <v>32825</v>
       </c>
-      <c r="O10" s="162"/>
-      <c r="P10" s="163"/>
+      <c r="O10" s="160"/>
+      <c r="P10" s="161"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="63"/>
       <c r="S10" s="6"/>
       <c r="T10" s="6"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.75">
-      <c r="A11" s="199"/>
+      <c r="A11" s="175"/>
       <c r="B11" s="18" t="s">
         <v>70</v>
       </c>
@@ -4125,33 +4125,33 @@
         <v>33233.199999999997</v>
       </c>
       <c r="G11" s="54"/>
-      <c r="H11" s="164" t="s">
+      <c r="H11" s="207" t="s">
         <v>71</v>
       </c>
-      <c r="I11" s="165"/>
-      <c r="J11" s="166">
+      <c r="I11" s="208"/>
+      <c r="J11" s="209">
         <f>B5</f>
         <v>656500</v>
       </c>
-      <c r="K11" s="167"/>
-      <c r="L11" s="168">
+      <c r="K11" s="210"/>
+      <c r="L11" s="211">
         <f>0.01507*C29</f>
         <v>1.5965858897603692E-2</v>
       </c>
-      <c r="M11" s="169"/>
-      <c r="N11" s="162">
+      <c r="M11" s="212"/>
+      <c r="N11" s="160">
         <f>L11*J11</f>
         <v>10481.586366276824</v>
       </c>
-      <c r="O11" s="162"/>
-      <c r="P11" s="163"/>
+      <c r="O11" s="160"/>
+      <c r="P11" s="161"/>
       <c r="Q11" s="61"/>
       <c r="R11" s="64"/>
       <c r="S11" s="6"/>
       <c r="T11" s="6"/>
     </row>
     <row r="12" spans="1:20" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A12" s="199"/>
+      <c r="A12" s="175"/>
       <c r="B12" s="18" t="s">
         <v>72</v>
       </c>
@@ -4169,27 +4169,27 @@
         <v>143000</v>
       </c>
       <c r="G12" s="6"/>
-      <c r="H12" s="186" t="s">
+      <c r="H12" s="162" t="s">
         <v>73</v>
       </c>
-      <c r="I12" s="187"/>
-      <c r="J12" s="187"/>
-      <c r="K12" s="187"/>
-      <c r="L12" s="187"/>
-      <c r="M12" s="188"/>
-      <c r="N12" s="189">
+      <c r="I12" s="163"/>
+      <c r="J12" s="163"/>
+      <c r="K12" s="163"/>
+      <c r="L12" s="163"/>
+      <c r="M12" s="164"/>
+      <c r="N12" s="165">
         <f>SUM(N8:P11)*(1+J5)</f>
         <v>502591.74500290456</v>
       </c>
-      <c r="O12" s="190"/>
-      <c r="P12" s="191"/>
+      <c r="O12" s="166"/>
+      <c r="P12" s="167"/>
       <c r="Q12" s="6"/>
       <c r="R12" s="64"/>
       <c r="S12" s="65"/>
       <c r="T12" s="6"/>
     </row>
     <row r="13" spans="1:20" ht="16.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A13" s="214"/>
+      <c r="A13" s="190"/>
       <c r="B13" s="19" t="s">
         <v>74</v>
       </c>
@@ -4240,20 +4240,20 @@
         <v>165880</v>
       </c>
       <c r="G14" s="6"/>
-      <c r="H14" s="192" t="s">
+      <c r="H14" s="168" t="s">
         <v>76</v>
       </c>
-      <c r="I14" s="193"/>
-      <c r="J14" s="193"/>
-      <c r="K14" s="193"/>
-      <c r="L14" s="193"/>
-      <c r="M14" s="194"/>
-      <c r="N14" s="195">
+      <c r="I14" s="169"/>
+      <c r="J14" s="169"/>
+      <c r="K14" s="169"/>
+      <c r="L14" s="169"/>
+      <c r="M14" s="170"/>
+      <c r="N14" s="171">
         <f>SUM(L8:M11)*(1+J5)</f>
         <v>0.76556244478736424</v>
       </c>
-      <c r="O14" s="196"/>
-      <c r="P14" s="197"/>
+      <c r="O14" s="172"/>
+      <c r="P14" s="173"/>
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="66"/>
@@ -4293,7 +4293,7 @@
       <c r="T15" s="6"/>
     </row>
     <row r="16" spans="1:20" ht="16.25" thickTop="1" x14ac:dyDescent="0.75">
-      <c r="A16" s="198" t="s">
+      <c r="A16" s="174" t="s">
         <v>78</v>
       </c>
       <c r="B16" s="17" t="s">
@@ -4313,27 +4313,27 @@
         <v>60060</v>
       </c>
       <c r="G16" s="6"/>
-      <c r="H16" s="201" t="s">
+      <c r="H16" s="177" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="202"/>
-      <c r="J16" s="202"/>
-      <c r="K16" s="202"/>
-      <c r="L16" s="202"/>
-      <c r="M16" s="203"/>
-      <c r="N16" s="204">
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="178"/>
+      <c r="L16" s="178"/>
+      <c r="M16" s="179"/>
+      <c r="N16" s="180">
         <f>N14+(F21/B5)</f>
         <v>2.4508169763943712</v>
       </c>
-      <c r="O16" s="205"/>
-      <c r="P16" s="206"/>
+      <c r="O16" s="181"/>
+      <c r="P16" s="182"/>
       <c r="Q16" s="6"/>
       <c r="R16" s="6"/>
       <c r="S16" s="6"/>
       <c r="T16" s="6"/>
     </row>
     <row r="17" spans="1:20" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A17" s="199"/>
+      <c r="A17" s="175"/>
       <c r="B17" s="18" t="s">
         <v>81</v>
       </c>
@@ -4351,29 +4351,29 @@
         <v>22880</v>
       </c>
       <c r="G17" s="6"/>
-      <c r="H17" s="210" t="s">
+      <c r="H17" s="186" t="s">
         <v>82</v>
       </c>
-      <c r="I17" s="211"/>
-      <c r="J17" s="212">
+      <c r="I17" s="187"/>
+      <c r="J17" s="188">
         <f>B5</f>
         <v>656500</v>
       </c>
-      <c r="K17" s="211"/>
+      <c r="K17" s="187"/>
       <c r="L17" s="58" t="s">
         <v>83</v>
       </c>
       <c r="M17" s="59"/>
-      <c r="N17" s="207"/>
-      <c r="O17" s="208"/>
-      <c r="P17" s="209"/>
+      <c r="N17" s="183"/>
+      <c r="O17" s="184"/>
+      <c r="P17" s="185"/>
       <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
     </row>
     <row r="18" spans="1:20" ht="16.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A18" s="200"/>
+      <c r="A18" s="176"/>
       <c r="B18" s="22" t="s">
         <v>84</v>
       </c>
@@ -4406,7 +4406,7 @@
       <c r="T18" s="6"/>
     </row>
     <row r="19" spans="1:20" ht="15.5" thickTop="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="183" t="s">
+      <c r="A19" s="157" t="s">
         <v>85</v>
       </c>
       <c r="B19" s="23" t="s">
@@ -4441,7 +4441,7 @@
       <c r="T19" s="6"/>
     </row>
     <row r="20" spans="1:20" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A20" s="184"/>
+      <c r="A20" s="158"/>
       <c r="B20" s="24" t="s">
         <v>87</v>
       </c>
@@ -4459,19 +4459,19 @@
         <v>0</v>
       </c>
       <c r="G20" s="6"/>
-      <c r="H20" s="185"/>
-      <c r="I20" s="185"/>
-      <c r="J20" s="185"/>
-      <c r="K20" s="185"/>
-      <c r="L20" s="185"/>
-      <c r="M20" s="185"/>
-      <c r="N20" s="185"/>
-      <c r="O20" s="185"/>
-      <c r="P20" s="185"/>
-      <c r="Q20" s="185"/>
-      <c r="R20" s="185"/>
-      <c r="S20" s="185"/>
-      <c r="T20" s="185"/>
+      <c r="H20" s="159"/>
+      <c r="I20" s="159"/>
+      <c r="J20" s="159"/>
+      <c r="K20" s="159"/>
+      <c r="L20" s="159"/>
+      <c r="M20" s="159"/>
+      <c r="N20" s="159"/>
+      <c r="O20" s="159"/>
+      <c r="P20" s="159"/>
+      <c r="Q20" s="159"/>
+      <c r="R20" s="159"/>
+      <c r="S20" s="159"/>
+      <c r="T20" s="159"/>
     </row>
     <row r="21" spans="1:20" ht="16.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A21" s="9" t="s">
@@ -4486,19 +4486,19 @@
         <v>1106369.6000000001</v>
       </c>
       <c r="G21" s="6"/>
-      <c r="H21" s="185"/>
-      <c r="I21" s="185"/>
-      <c r="J21" s="185"/>
-      <c r="K21" s="185"/>
-      <c r="L21" s="185"/>
-      <c r="M21" s="185"/>
-      <c r="N21" s="185"/>
-      <c r="O21" s="185"/>
-      <c r="P21" s="185"/>
-      <c r="Q21" s="185"/>
-      <c r="R21" s="185"/>
-      <c r="S21" s="185"/>
-      <c r="T21" s="185"/>
+      <c r="H21" s="159"/>
+      <c r="I21" s="159"/>
+      <c r="J21" s="159"/>
+      <c r="K21" s="159"/>
+      <c r="L21" s="159"/>
+      <c r="M21" s="159"/>
+      <c r="N21" s="159"/>
+      <c r="O21" s="159"/>
+      <c r="P21" s="159"/>
+      <c r="Q21" s="159"/>
+      <c r="R21" s="159"/>
+      <c r="S21" s="159"/>
+      <c r="T21" s="159"/>
     </row>
     <row r="22" spans="1:20" ht="15.5" thickTop="1" x14ac:dyDescent="0.75">
       <c r="A22" s="10" t="s">
@@ -4718,6 +4718,24 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="H20:T21"/>
     <mergeCell ref="N11:P11"/>
@@ -4734,24 +4752,6 @@
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="L8:M8"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:P9"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Costs per dog vaccinated" prompt="Enter the estimated cost per dog vaccinated.  Costs are presented in USD, therefore user will need to convert into their local currency. " sqref="B5" xr:uid="{69D90B4D-BC64-4C0C-9B68-3F349EA33EB4}"/>

</xml_diff>